<commit_message>
Patch 6 test on server - Kegg debug
</commit_message>
<xml_diff>
--- a/data/metadata/metadata.xlsx
+++ b/data/metadata/metadata.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MicrobExplorer\data\metadata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yanni\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{77BDE310-B9A3-49C1-A896-80A1E972B741}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3B99012-E26D-4C6B-ADD9-784C902815D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{1D82295F-C9E4-41E4-8467-00986F3B4F5E}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="46">
   <si>
     <t>sample_id</t>
   </si>
@@ -99,9 +99,6 @@
     <t>TD6</t>
   </si>
   <si>
-    <t>TD1_250810</t>
-  </si>
-  <si>
     <t>TD1_251015</t>
   </si>
   <si>
@@ -111,9 +108,6 @@
     <t>TD1_251029</t>
   </si>
   <si>
-    <t>TD2_250810</t>
-  </si>
-  <si>
     <t>TD2_251015</t>
   </si>
   <si>
@@ -123,9 +117,6 @@
     <t>TD2_251029</t>
   </si>
   <si>
-    <t>TD3_250810</t>
-  </si>
-  <si>
     <t>TD3_251015</t>
   </si>
   <si>
@@ -135,9 +126,6 @@
     <t>TD3_251029</t>
   </si>
   <si>
-    <t>TD4_250810</t>
-  </si>
-  <si>
     <t>TD4_251015</t>
   </si>
   <si>
@@ -147,9 +135,6 @@
     <t>TD4_251029</t>
   </si>
   <si>
-    <t>TD5_250810</t>
-  </si>
-  <si>
     <t>TD5_251015</t>
   </si>
   <si>
@@ -159,9 +144,6 @@
     <t>TD5_251029</t>
   </si>
   <si>
-    <t>TD6_250810</t>
-  </si>
-  <si>
     <t>TD6_251015</t>
   </si>
   <si>
@@ -169,6 +151,27 @@
   </si>
   <si>
     <t>TD6_251029</t>
+  </si>
+  <si>
+    <t>TD5_251008</t>
+  </si>
+  <si>
+    <t>TD6_251008</t>
+  </si>
+  <si>
+    <t>TD4_251008</t>
+  </si>
+  <si>
+    <t>TD3_251008</t>
+  </si>
+  <si>
+    <t>TD2_251008</t>
+  </si>
+  <si>
+    <t>TD1_251008</t>
+  </si>
+  <si>
+    <t>group</t>
   </si>
 </sst>
 </file>
@@ -521,413 +524,524 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7072A79C-54ED-44A8-82C9-639E3038EC67}">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="1">
         <v>45875</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="1">
+        <v>45879</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="1">
+        <v>45883</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>21</v>
       </c>
-      <c r="B3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="1">
-        <v>45879</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="1">
-        <v>45883</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="1">
+        <v>45945</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>22</v>
       </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="1">
-        <v>45945</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="1">
+        <v>45952</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>23</v>
       </c>
-      <c r="B6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="1">
-        <v>45952</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>24</v>
-      </c>
       <c r="B7" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="1">
         <v>45959</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
       <c r="B8" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" s="1">
         <v>45875</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="1">
+        <v>45879</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" s="1">
+        <v>45883</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" s="1">
+        <v>45945</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>25</v>
       </c>
-      <c r="B9" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="1">
-        <v>45879</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>6</v>
-      </c>
-      <c r="B10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" s="1">
-        <v>45883</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="B12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" s="1">
+        <v>45952</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>26</v>
       </c>
-      <c r="B11" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11" s="1">
-        <v>45945</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" s="1">
-        <v>45952</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>28</v>
-      </c>
       <c r="B13" t="s">
         <v>16</v>
       </c>
-      <c r="C13" s="1">
+      <c r="C13" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" s="1">
         <v>45959</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>7</v>
       </c>
       <c r="B14" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="1">
+      <c r="C14" t="s">
+        <v>17</v>
+      </c>
+      <c r="D14" s="1">
         <v>45875</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" t="s">
+        <v>17</v>
+      </c>
+      <c r="D15" s="1">
+        <v>45879</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D16" s="1">
+        <v>45883</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" t="s">
+        <v>17</v>
+      </c>
+      <c r="C17" t="s">
+        <v>17</v>
+      </c>
+      <c r="D17" s="1">
+        <v>45945</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>28</v>
+      </c>
+      <c r="B18" t="s">
+        <v>17</v>
+      </c>
+      <c r="C18" t="s">
+        <v>17</v>
+      </c>
+      <c r="D18" s="1">
+        <v>45952</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>29</v>
       </c>
-      <c r="B15" t="s">
-        <v>17</v>
-      </c>
-      <c r="C15" s="1">
-        <v>45879</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>8</v>
-      </c>
-      <c r="B16" t="s">
-        <v>17</v>
-      </c>
-      <c r="C16" s="1">
-        <v>45883</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>30</v>
-      </c>
-      <c r="B17" t="s">
-        <v>17</v>
-      </c>
-      <c r="C17" s="1">
-        <v>45945</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>31</v>
-      </c>
-      <c r="B18" t="s">
-        <v>17</v>
-      </c>
-      <c r="C18" s="1">
-        <v>45952</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>32</v>
-      </c>
       <c r="B19" t="s">
         <v>17</v>
       </c>
-      <c r="C19" s="1">
+      <c r="C19" t="s">
+        <v>17</v>
+      </c>
+      <c r="D19" s="1">
         <v>45959</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>9</v>
       </c>
       <c r="B20" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="1">
+      <c r="C20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D20" s="1">
         <v>45875</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="B21" t="s">
         <v>18</v>
       </c>
-      <c r="C21" s="1">
+      <c r="C21" t="s">
+        <v>18</v>
+      </c>
+      <c r="D21" s="1">
         <v>45879</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="B22" t="s">
         <v>18</v>
       </c>
-      <c r="C22" s="1">
+      <c r="C22" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="1">
         <v>45883</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B23" t="s">
         <v>18</v>
       </c>
-      <c r="C23" s="1">
+      <c r="C23" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" s="1">
         <v>45945</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B24" t="s">
         <v>18</v>
       </c>
-      <c r="C24" s="1">
+      <c r="C24" t="s">
+        <v>18</v>
+      </c>
+      <c r="D24" s="1">
         <v>45952</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B25" t="s">
         <v>18</v>
       </c>
-      <c r="C25" s="1">
+      <c r="C25" t="s">
+        <v>18</v>
+      </c>
+      <c r="D25" s="1">
         <v>45959</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>11</v>
       </c>
       <c r="B26" t="s">
         <v>19</v>
       </c>
-      <c r="C26" s="1">
+      <c r="C26" t="s">
+        <v>19</v>
+      </c>
+      <c r="D26" s="1">
         <v>45875</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="B27" t="s">
         <v>19</v>
       </c>
-      <c r="C27" s="1">
+      <c r="C27" t="s">
+        <v>19</v>
+      </c>
+      <c r="D27" s="1">
         <v>45879</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="B28" t="s">
         <v>19</v>
       </c>
-      <c r="C28" s="1">
+      <c r="C28" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" s="1">
         <v>45883</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B29" t="s">
         <v>19</v>
       </c>
-      <c r="C29" s="1">
+      <c r="C29" t="s">
+        <v>19</v>
+      </c>
+      <c r="D29" s="1">
         <v>45945</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B30" t="s">
         <v>19</v>
       </c>
-      <c r="C30" s="1">
+      <c r="C30" t="s">
+        <v>19</v>
+      </c>
+      <c r="D30" s="1">
         <v>45952</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B31" t="s">
         <v>19</v>
       </c>
-      <c r="C31" s="1">
+      <c r="C31" t="s">
+        <v>19</v>
+      </c>
+      <c r="D31" s="1">
         <v>45959</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>13</v>
       </c>
       <c r="B32" t="s">
         <v>20</v>
       </c>
-      <c r="C32" s="1">
+      <c r="C32" t="s">
+        <v>20</v>
+      </c>
+      <c r="D32" s="1">
         <v>45875</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="B33" t="s">
         <v>20</v>
       </c>
-      <c r="C33" s="1">
+      <c r="C33" t="s">
+        <v>20</v>
+      </c>
+      <c r="D33" s="1">
         <v>45879</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="B34" t="s">
         <v>20</v>
       </c>
-      <c r="C34" s="1">
+      <c r="C34" t="s">
+        <v>20</v>
+      </c>
+      <c r="D34" s="1">
         <v>45883</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B35" t="s">
         <v>20</v>
       </c>
-      <c r="C35" s="1">
+      <c r="C35" t="s">
+        <v>20</v>
+      </c>
+      <c r="D35" s="1">
         <v>45945</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="B36" t="s">
         <v>20</v>
       </c>
-      <c r="C36" s="1">
+      <c r="C36" t="s">
+        <v>20</v>
+      </c>
+      <c r="D36" s="1">
         <v>45952</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="B37" t="s">
         <v>20</v>
       </c>
-      <c r="C37" s="1">
+      <c r="C37" t="s">
+        <v>20</v>
+      </c>
+      <c r="D37" s="1">
         <v>45959</v>
       </c>
     </row>

</xml_diff>